<commit_message>
Add eSimConfig install/delete gap to developer schema-update sheet
Row 5: eSimConfig is missing install and delete payloads (only get/set
exist on both channels) — request the developer to add them to the schema.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RestAPI/developer_feedback/schema_update_requests.xlsx
+++ b/RestAPI/developer_feedback/schema_update_requests.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -747,6 +747,52 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="88" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>eSIM configuration</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>REST: /cloud/eSimConfig (getEsimConfig, setEsimConfig)
+MQTT: get_eSimConfig, set_eSimConfig</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>The eSimConfig API is missing the install and delete payloads. Only get and set operations are currently defined.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Add the install and delete payloads (operations) for eSimConfig.</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Payloads: Install, Delete</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Currently only get/set eSimConfig exist on both channels. Please add the install and delete payloads to the schema.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>

</xml_diff>